<commit_message>
Flag Selwyn Contractors (HH001) as arrears; store signed lease agreement
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wwD7VViSS7KiZMtmdgnsd
</commit_message>
<xml_diff>
--- a/data/HireHospo_Database.xlsx
+++ b/data/HireHospo_Database.xlsx
@@ -465,10 +465,14 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="n"/>
+          <t>arrears</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Signed Lease-For-Ownership (36m) proposal 9/9/2025. Legal entity: SELWYN CONTRACTORS LIMITED (8761910). NON-PAYING - in arrears (owner confirmed 19/07/2026). Contract PDF: data/contracts/SELWYN_CONTRACTORS_lease_agreement.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>